<commit_message>
feat: add template file for group registration in public assets
</commit_message>
<xml_diff>
--- a/client/public/plantilla_inscripcion_grupos.xlsx
+++ b/client/public/plantilla_inscripcion_grupos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,22 +456,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>perfil</t>
+          <t>institucion</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>institucion</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
           <t>carrera</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>comision</t>
         </is>
       </c>
     </row>
@@ -503,22 +493,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>STUDENT</t>
+          <t>UNAB</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>UNAB</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
           <t>Lic. en Logística</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Comisión A - Turno Noche</t>
         </is>
       </c>
     </row>
@@ -550,22 +530,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>VISITOR</t>
+          <t>Instituto Belgrano</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Instituto Belgrano</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
           <t>Tecnico Superior</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>6to Año - Division B</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement backend diagnostic scripts, registration serializers, and alert verification tools while updating gitignore rules
</commit_message>
<xml_diff>
--- a/client/public/plantilla_inscripcion_grupos.xlsx
+++ b/client/public/plantilla_inscripcion_grupos.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,43 +425,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>nombre</t>
+          <t>Nombre</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>apellido</t>
+          <t>Apellido</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>DNI</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>dni</t>
+          <t>Celular</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>telefono</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>institucion</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>carrera</t>
+          <t>Email</t>
         </is>
       </c>
     </row>
@@ -473,69 +463,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Pérez</t>
+          <t>Perez</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1122334455</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>juan.perez@ejemplo.com</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>12345678</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1122334455</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>UNAB</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Lic. en Logística</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Ana</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>García</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>ana.garcia@ejemplo.com</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>87654321</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1166778899</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Instituto Belgrano</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Tecnico Superior</t>
         </is>
       </c>
     </row>

</xml_diff>